<commit_message>
res + model comparison
</commit_message>
<xml_diff>
--- a/source/CP/Before_Circle/model_comparison_14.xlsx
+++ b/source/CP/Before_Circle/model_comparison_14.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xPica\Documents\CDMO_Proj_LiPiDo\source\CP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xPica\Documents\CDMO_Proj_LiPiDo\source\CP\Before_Circle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4673E7C4-21F0-4CB1-A6F1-BAA5BD6D3BDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E23AE48-93A0-4F76-892D-71EE28DD5AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -186,18 +186,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -215,16 +214,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -528,13 +517,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T32"/>
+  <dimension ref="A1:R32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="14" max="14" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -572,7 +561,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -614,7 +603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -656,7 +645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -698,7 +687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -740,7 +729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -781,8 +770,9 @@
       <c r="N6" t="b">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="O6" s="2"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -823,9 +813,8 @@
       <c r="N7" t="b">
         <v>0</v>
       </c>
-      <c r="T7" s="3"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -866,9 +855,8 @@
       <c r="N8" t="b">
         <v>0</v>
       </c>
-      <c r="R8" s="3"/>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -910,7 +898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -952,7 +940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -994,7 +982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1036,7 +1024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1078,7 +1066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1120,7 +1108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1162,7 +1150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1220,7 +1208,6 @@
       <c r="C19">
         <v>2.5124000000000001E-3</v>
       </c>
-      <c r="H19" s="3"/>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B20">
@@ -1229,7 +1216,6 @@
       <c r="C20">
         <v>1.0574E-3</v>
       </c>
-      <c r="K20" s="3"/>
     </row>
     <row r="21" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B21">
@@ -1328,21 +1314,8 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J2:K16">
-    <cfRule type="cellIs" dxfId="2" priority="5" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:E16 M2:N16 J2:K16 G2:H16">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
-      <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
-      <formula>FALSE</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L16 F2:F16 I2:I16 C2:C16">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="B18:C32">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1353,8 +1326,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B18:C32">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="D2:E16 G2:H16 J2:K16 M2:N16">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+      <formula>TRUE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+      <formula>FALSE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L16 F2:F16 I2:I16 C2:C16">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>